<commit_message>
Rechendurchläufe und _Modellanpassungen - Sensitivitäten
</commit_message>
<xml_diff>
--- a/FischerTropsch_Paper/Patagonien_FischerTropsch_3_Naphta_Bio_Brownfield_MH/Datenbank.xlsx
+++ b/FischerTropsch_Paper/Patagonien_FischerTropsch_3_Naphta_Bio_Brownfield_MH/Datenbank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hem38994\Documents\GitHub\FENES_P2X\FischerTropsch_Paper_Michi\Patagonien_FischerTropsch_3_Naphta_Bio_Brownfield_MH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hem38994\Documents\GitHub\FENES_P2X\FischerTropsch_Paper\Patagonien_FischerTropsch_3_Naphta_Bio_Brownfield_MH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E19BE4A6-0EDF-4943-87CD-05EAE8216912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D69A7EB-6537-4D7D-93A7-3A80136127E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4455" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-6945" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -162,7 +162,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="405">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -1373,6 +1373,12 @@
   </si>
   <si>
     <t>€/ kg a</t>
+  </si>
+  <si>
+    <t>Landesspezifischer Zinssatz</t>
+  </si>
+  <si>
+    <t>wacc_change</t>
   </si>
 </sst>
 </file>
@@ -1633,11 +1639,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1965,24 +1971,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G78"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G79"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" style="24" customWidth="1"/>
-    <col min="3" max="3" width="36.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6328125" style="24" customWidth="1"/>
+    <col min="3" max="3" width="36.1796875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="11" max="11" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="21" t="s">
         <v>69</v>
       </c>
@@ -2003,7 +2009,7 @@
       </c>
       <c r="G1" s="24"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="40" t="s">
         <v>70</v>
       </c>
@@ -2023,7 +2029,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="41"/>
       <c r="B3" s="48"/>
       <c r="C3" s="1" t="s">
@@ -2039,7 +2045,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="41"/>
       <c r="B4" s="48"/>
       <c r="C4" s="1" t="s">
@@ -2055,7 +2061,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="41"/>
       <c r="B5" s="48"/>
       <c r="C5" s="1" t="s">
@@ -2071,7 +2077,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="41"/>
       <c r="B6" s="48"/>
       <c r="C6" s="1" t="s">
@@ -2087,7 +2093,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="41"/>
       <c r="B7" s="48"/>
       <c r="C7" s="1" t="s">
@@ -2103,7 +2109,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="41"/>
       <c r="B8" s="51" t="s">
         <v>299</v>
@@ -2121,7 +2127,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="41"/>
       <c r="B9" s="48"/>
       <c r="C9" s="1" t="s">
@@ -2137,7 +2143,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="41"/>
       <c r="B10" s="48"/>
       <c r="C10" s="1" t="s">
@@ -2153,7 +2159,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="41"/>
       <c r="B11" s="48"/>
       <c r="C11" s="1" t="s">
@@ -2169,7 +2175,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="41"/>
       <c r="B12" s="48"/>
       <c r="C12" s="1" t="s">
@@ -2185,7 +2191,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="41"/>
       <c r="B13" s="48"/>
       <c r="C13" s="1" t="s">
@@ -2201,7 +2207,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="41"/>
       <c r="B14" s="48"/>
       <c r="C14" s="1" t="s">
@@ -2217,7 +2223,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="41"/>
       <c r="B15" s="48"/>
       <c r="C15" s="1" t="s">
@@ -2233,7 +2239,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="41"/>
       <c r="B16" s="52"/>
       <c r="C16" s="17" t="s">
@@ -2249,7 +2255,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="41"/>
       <c r="B17" s="51" t="s">
         <v>236</v>
@@ -2267,7 +2273,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="41"/>
       <c r="B18" s="48"/>
       <c r="C18" s="1" t="s">
@@ -2283,7 +2289,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="41"/>
       <c r="B19" s="48"/>
       <c r="C19" s="1" t="s">
@@ -2299,7 +2305,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="41"/>
       <c r="B20" s="48"/>
       <c r="C20" s="1" t="s">
@@ -2315,7 +2321,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="41"/>
       <c r="B21" s="48"/>
       <c r="C21" s="1" t="s">
@@ -2331,7 +2337,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="41"/>
       <c r="B22" s="52"/>
       <c r="C22" s="17" t="s">
@@ -2347,7 +2353,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="41"/>
       <c r="B23" s="39" t="s">
         <v>382</v>
@@ -2365,7 +2371,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="41"/>
       <c r="B24" s="39"/>
       <c r="C24" s="1" t="s">
@@ -2381,7 +2387,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="41"/>
       <c r="B25" s="39"/>
       <c r="C25" s="1" t="s">
@@ -2397,7 +2403,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="41"/>
       <c r="B26" s="39"/>
       <c r="C26" s="1" t="s">
@@ -2413,7 +2419,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="41"/>
       <c r="B27" s="39"/>
       <c r="C27" s="1" t="s">
@@ -2429,7 +2435,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="41"/>
       <c r="B28" s="39"/>
       <c r="C28" s="1" t="s">
@@ -2445,7 +2451,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="41"/>
       <c r="B29" s="39"/>
       <c r="C29" s="1" t="s">
@@ -2461,7 +2467,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="41"/>
       <c r="B30" s="39"/>
       <c r="C30" s="1" t="s">
@@ -2477,7 +2483,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="41"/>
       <c r="B31" s="39"/>
       <c r="C31" s="1" t="s">
@@ -2493,7 +2499,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="40" t="s">
         <v>71</v>
       </c>
@@ -2513,7 +2519,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="41"/>
       <c r="B33" s="44"/>
       <c r="C33" s="1" t="s">
@@ -2529,7 +2535,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="41"/>
       <c r="B34" s="44"/>
       <c r="C34" s="1" t="s">
@@ -2545,7 +2551,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="41"/>
       <c r="B35" s="44"/>
       <c r="C35" s="1" t="s">
@@ -2561,7 +2567,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="41"/>
       <c r="B36" s="44"/>
       <c r="C36" s="1" t="s">
@@ -2577,7 +2583,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="41"/>
       <c r="B37" s="44"/>
       <c r="C37" s="1" t="s">
@@ -2593,7 +2599,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="41"/>
       <c r="B38" s="44"/>
       <c r="C38" s="1" t="s">
@@ -2609,7 +2615,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="41"/>
       <c r="B39" s="45"/>
       <c r="C39" s="17" t="s">
@@ -2625,7 +2631,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="41"/>
       <c r="B40" s="46" t="s">
         <v>274</v>
@@ -2643,7 +2649,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="41"/>
       <c r="B41" s="44"/>
       <c r="C41" s="1" t="s">
@@ -2659,7 +2665,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="41"/>
       <c r="B42" s="44"/>
       <c r="C42" s="1" t="s">
@@ -2675,7 +2681,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="41"/>
       <c r="B43" s="44"/>
       <c r="C43" s="1" t="s">
@@ -2691,7 +2697,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="41"/>
       <c r="B44" s="44"/>
       <c r="C44" s="1" t="s">
@@ -2707,7 +2713,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="41"/>
       <c r="B45" s="44"/>
       <c r="C45" s="1" t="s">
@@ -2723,7 +2729,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="41"/>
       <c r="B46" s="44"/>
       <c r="C46" s="1" t="s">
@@ -2739,7 +2745,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="41"/>
       <c r="B47" s="44"/>
       <c r="C47" s="17" t="s">
@@ -2755,7 +2761,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="41"/>
       <c r="B48" s="46" t="s">
         <v>201</v>
@@ -2773,7 +2779,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="41"/>
       <c r="B49" s="48"/>
       <c r="C49" s="1" t="s">
@@ -2790,7 +2796,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="41"/>
       <c r="B50" s="48"/>
       <c r="C50" s="1" t="s">
@@ -2806,7 +2812,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="41"/>
       <c r="B51" s="48"/>
       <c r="C51" s="1" t="s">
@@ -2822,7 +2828,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="41"/>
       <c r="B52" s="48"/>
       <c r="C52" s="1" t="s">
@@ -2838,7 +2844,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="41"/>
       <c r="B53" s="48"/>
       <c r="C53" s="1" t="s">
@@ -2854,7 +2860,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="41"/>
       <c r="B54" s="48"/>
       <c r="C54" s="1" t="s">
@@ -2870,7 +2876,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="41"/>
       <c r="B55" s="48"/>
       <c r="C55" s="1" t="s">
@@ -2886,7 +2892,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="41"/>
       <c r="B56" s="48"/>
       <c r="C56" s="1" t="s">
@@ -2902,7 +2908,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="42"/>
       <c r="B57" s="49"/>
       <c r="C57" s="27" t="s">
@@ -2918,7 +2924,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="40" t="s">
         <v>72</v>
       </c>
@@ -2938,7 +2944,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="41"/>
       <c r="B59" s="36" t="s">
         <v>376</v>
@@ -2956,7 +2962,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="41"/>
       <c r="B60" s="46" t="s">
         <v>4</v>
@@ -2974,7 +2980,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="41"/>
       <c r="B61" s="44"/>
       <c r="C61" s="1" t="s">
@@ -2990,7 +2996,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="41"/>
       <c r="B62" s="44"/>
       <c r="C62" s="1" t="s">
@@ -3006,7 +3012,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="41"/>
       <c r="B63" s="44"/>
       <c r="C63" s="1" t="s">
@@ -3022,7 +3028,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="41"/>
       <c r="B64" s="44"/>
       <c r="C64" s="1" t="s">
@@ -3038,7 +3044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="41"/>
       <c r="B65" s="44"/>
       <c r="C65" s="1" t="s">
@@ -3054,7 +3060,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="41"/>
       <c r="B66" s="45"/>
       <c r="C66" s="17" t="s">
@@ -3070,7 +3076,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="41"/>
       <c r="B67" s="46" t="s">
         <v>5</v>
@@ -3088,7 +3094,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="41"/>
       <c r="B68" s="44"/>
       <c r="C68" s="1" t="s">
@@ -3104,7 +3110,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="41"/>
       <c r="B69" s="44"/>
       <c r="C69" s="1" t="s">
@@ -3120,7 +3126,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="41"/>
       <c r="B70" s="44"/>
       <c r="C70" s="1" t="s">
@@ -3136,7 +3142,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="41"/>
       <c r="B71" s="44"/>
       <c r="C71" s="1" t="s">
@@ -3152,7 +3158,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="41"/>
       <c r="B72" s="44"/>
       <c r="C72" s="1" t="s">
@@ -3168,7 +3174,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="42"/>
       <c r="B73" s="47"/>
       <c r="C73" s="27" t="s">
@@ -3184,7 +3190,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="40" t="s">
         <v>76</v>
       </c>
@@ -3204,7 +3210,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="41"/>
       <c r="B75" s="24" t="s">
         <v>259</v>
@@ -3222,7 +3228,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="41"/>
       <c r="B76" s="33" t="s">
         <v>79</v>
@@ -3240,7 +3246,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="41"/>
       <c r="B77" s="33" t="s">
         <v>340</v>
@@ -3258,7 +3264,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="42"/>
       <c r="B78" s="22" t="s">
         <v>300</v>
@@ -3275,6 +3281,26 @@
       </c>
       <c r="F78" s="27" t="s">
         <v>314</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B79" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E79" s="3">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3302,18 +3328,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AB2E79-6F94-41B5-A552-C40EC4890194}">
   <dimension ref="A1:F152"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="50.77734375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="46.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.5546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.5546875" style="1"/>
+    <col min="1" max="1" width="14.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.81640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="46.08984375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.54296875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.54296875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="21" t="s">
         <v>69</v>
       </c>
@@ -3333,7 +3359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="40" t="s">
         <v>70</v>
       </c>
@@ -3351,7 +3377,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="41"/>
       <c r="B3" s="48"/>
       <c r="C3" s="1" t="s">
@@ -3365,7 +3391,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="41"/>
       <c r="B4" s="48"/>
       <c r="C4" s="1" t="s">
@@ -3379,7 +3405,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="41"/>
       <c r="B5" s="48"/>
       <c r="C5" s="1" t="s">
@@ -3393,7 +3419,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="41"/>
       <c r="B6" s="48"/>
       <c r="C6" s="1" t="s">
@@ -3407,7 +3433,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="41"/>
       <c r="B7" s="48"/>
       <c r="C7" s="1" t="s">
@@ -3421,7 +3447,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="41"/>
       <c r="B8" s="48"/>
       <c r="C8" s="1" t="s">
@@ -3435,7 +3461,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="41"/>
       <c r="B9" s="48"/>
       <c r="C9" s="1" t="s">
@@ -3449,7 +3475,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="41"/>
       <c r="B10" s="48"/>
       <c r="C10" s="1" t="s">
@@ -3463,12 +3489,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="41"/>
       <c r="B11" s="48"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="41"/>
       <c r="B12" s="51" t="s">
         <v>333</v>
@@ -3484,7 +3510,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="41"/>
       <c r="B13" s="48"/>
       <c r="C13" s="1" t="s">
@@ -3498,7 +3524,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="41"/>
       <c r="B14" s="48"/>
       <c r="C14" s="1" t="s">
@@ -3512,7 +3538,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="41"/>
       <c r="B15" s="48"/>
       <c r="C15" s="1" t="s">
@@ -3526,7 +3552,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="41"/>
       <c r="B16" s="48"/>
       <c r="C16" s="1" t="s">
@@ -3540,7 +3566,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="41"/>
       <c r="B17" s="48"/>
       <c r="C17" s="1" t="s">
@@ -3554,7 +3580,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="41"/>
       <c r="B18" s="48"/>
       <c r="C18" s="1" t="s">
@@ -3568,7 +3594,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="41"/>
       <c r="B19" s="48"/>
       <c r="C19" s="1" t="s">
@@ -3582,7 +3608,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="41"/>
       <c r="B20" s="48"/>
       <c r="C20" s="1" t="s">
@@ -3596,7 +3622,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="41"/>
       <c r="B21" s="48"/>
       <c r="C21" s="1" t="s">
@@ -3610,7 +3636,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="41"/>
       <c r="B22" s="48"/>
       <c r="C22" s="1" t="s">
@@ -3624,7 +3650,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="41"/>
       <c r="B23" s="52"/>
       <c r="C23" s="17"/>
@@ -3632,7 +3658,7 @@
       <c r="E23" s="18"/>
       <c r="F23" s="17"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="41"/>
       <c r="B24" s="51" t="s">
         <v>236</v>
@@ -3648,7 +3674,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="41"/>
       <c r="B25" s="48"/>
       <c r="C25" s="1" t="s">
@@ -3662,7 +3688,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="41"/>
       <c r="B26" s="48"/>
       <c r="C26" s="1" t="s">
@@ -3676,7 +3702,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="41"/>
       <c r="B27" s="48"/>
       <c r="C27" s="1" t="s">
@@ -3690,7 +3716,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="41"/>
       <c r="B28" s="48"/>
       <c r="C28" s="1" t="s">
@@ -3704,7 +3730,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="41"/>
       <c r="B29" s="48"/>
       <c r="C29" s="1" t="s">
@@ -3718,7 +3744,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="41"/>
       <c r="B30" s="48"/>
       <c r="C30" s="1" t="s">
@@ -3732,7 +3758,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="41"/>
       <c r="B31" s="48"/>
       <c r="C31" s="1" t="s">
@@ -3746,7 +3772,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="41"/>
       <c r="B32" s="48"/>
       <c r="C32" s="1" t="s">
@@ -3760,7 +3786,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="41"/>
       <c r="B33" s="52"/>
       <c r="C33" s="17"/>
@@ -3768,7 +3794,7 @@
       <c r="E33" s="18"/>
       <c r="F33" s="17"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="41"/>
       <c r="B34" s="39" t="s">
         <v>361</v>
@@ -3784,7 +3810,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="41"/>
       <c r="B35" s="39"/>
       <c r="C35" s="1" t="s">
@@ -3798,7 +3824,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="41"/>
       <c r="B36" s="39"/>
       <c r="C36" s="1" t="s">
@@ -3812,7 +3838,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="41"/>
       <c r="B37" s="39"/>
       <c r="C37" s="1" t="s">
@@ -3826,7 +3852,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="41"/>
       <c r="B38" s="39"/>
       <c r="C38" s="1" t="s">
@@ -3840,7 +3866,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="41"/>
       <c r="B39" s="39"/>
       <c r="C39" s="1" t="s">
@@ -3854,7 +3880,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="41"/>
       <c r="B40" s="39"/>
       <c r="C40" s="1" t="s">
@@ -3868,7 +3894,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="41"/>
       <c r="B41" s="39"/>
       <c r="C41" s="1" t="s">
@@ -3882,7 +3908,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="41"/>
       <c r="B42" s="39"/>
       <c r="C42" s="1" t="s">
@@ -3896,7 +3922,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="41"/>
       <c r="B43" s="39"/>
       <c r="C43" s="1" t="s">
@@ -3910,7 +3936,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="41"/>
       <c r="B44" s="39"/>
       <c r="C44" s="1" t="s">
@@ -3924,7 +3950,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="41"/>
       <c r="B45" s="39"/>
       <c r="C45" s="1" t="s">
@@ -3938,12 +3964,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="41"/>
       <c r="B46" s="39"/>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="40" t="s">
         <v>71</v>
       </c>
@@ -3961,7 +3987,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="41"/>
       <c r="B48" s="44"/>
       <c r="C48" s="1" t="s">
@@ -3975,7 +4001,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="41"/>
       <c r="B49" s="44"/>
       <c r="C49" s="1" t="s">
@@ -3989,7 +4015,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="41"/>
       <c r="B50" s="44"/>
       <c r="C50" s="1" t="s">
@@ -4003,7 +4029,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="41"/>
       <c r="B51" s="44"/>
       <c r="C51" s="1" t="s">
@@ -4017,7 +4043,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="41"/>
       <c r="B52" s="44"/>
       <c r="C52" s="1" t="s">
@@ -4031,7 +4057,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="41"/>
       <c r="B53" s="44"/>
       <c r="C53" s="1" t="s">
@@ -4045,7 +4071,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="41"/>
       <c r="B54" s="44"/>
       <c r="C54" s="1" t="s">
@@ -4059,7 +4085,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="41"/>
       <c r="B55" s="44"/>
       <c r="C55" s="1" t="s">
@@ -4073,7 +4099,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="41"/>
       <c r="B56" s="45"/>
       <c r="C56" s="17"/>
@@ -4081,7 +4107,7 @@
       <c r="E56" s="18"/>
       <c r="F56" s="17"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="41"/>
       <c r="B57" s="44" t="s">
         <v>274</v>
@@ -4097,7 +4123,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="41"/>
       <c r="B58" s="44"/>
       <c r="C58" s="1" t="s">
@@ -4111,7 +4137,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="41"/>
       <c r="B59" s="44"/>
       <c r="C59" s="1" t="s">
@@ -4125,7 +4151,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="41"/>
       <c r="B60" s="44"/>
       <c r="C60" s="1" t="s">
@@ -4139,7 +4165,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="41"/>
       <c r="B61" s="44"/>
       <c r="C61" s="1" t="s">
@@ -4153,7 +4179,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="41"/>
       <c r="B62" s="44"/>
       <c r="C62" s="1" t="s">
@@ -4167,7 +4193,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="41"/>
       <c r="B63" s="44"/>
       <c r="C63" s="1" t="s">
@@ -4181,7 +4207,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="41"/>
       <c r="B64" s="44"/>
       <c r="C64" s="1" t="s">
@@ -4195,7 +4221,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="41"/>
       <c r="B65" s="44"/>
       <c r="C65" s="1" t="s">
@@ -4209,12 +4235,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="41"/>
       <c r="B66" s="45"/>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="41"/>
       <c r="B67" s="46" t="s">
         <v>6</v>
@@ -4230,7 +4256,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="41"/>
       <c r="B68" s="44"/>
       <c r="C68" s="1" t="s">
@@ -4244,7 +4270,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="41"/>
       <c r="B69" s="48"/>
       <c r="C69" s="1" t="s">
@@ -4258,7 +4284,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="41"/>
       <c r="B70" s="48"/>
       <c r="C70" s="1" t="s">
@@ -4272,7 +4298,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="41"/>
       <c r="B71" s="48"/>
       <c r="C71" s="1" t="s">
@@ -4286,7 +4312,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="41"/>
       <c r="B72" s="48"/>
       <c r="C72" s="1" t="s">
@@ -4300,7 +4326,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="41"/>
       <c r="B73" s="48"/>
       <c r="C73" s="1" t="s">
@@ -4314,7 +4340,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="41"/>
       <c r="B74" s="48"/>
       <c r="C74" s="1" t="s">
@@ -4328,7 +4354,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="41"/>
       <c r="B75" s="48"/>
       <c r="C75" s="1" t="s">
@@ -4342,7 +4368,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="41"/>
       <c r="B76" s="48"/>
       <c r="C76" s="1" t="s">
@@ -4356,7 +4382,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="41"/>
       <c r="B77" s="48"/>
       <c r="C77" s="1" t="s">
@@ -4370,7 +4396,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="42"/>
       <c r="B78" s="49"/>
       <c r="C78" s="27"/>
@@ -4378,7 +4404,7 @@
       <c r="E78" s="28"/>
       <c r="F78" s="27"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="40" t="s">
         <v>72</v>
       </c>
@@ -4396,7 +4422,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="41"/>
       <c r="B80" s="48"/>
       <c r="C80" s="1" t="s">
@@ -4410,7 +4436,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="41"/>
       <c r="B81" s="52"/>
       <c r="C81" s="17"/>
@@ -4418,9 +4444,9 @@
       <c r="E81" s="38"/>
       <c r="F81" s="17"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="41"/>
-      <c r="B82" s="53" t="s">
+      <c r="B82" s="54" t="s">
         <v>376</v>
       </c>
       <c r="C82" s="1" t="s">
@@ -4434,9 +4460,9 @@
         <v>379</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="41"/>
-      <c r="B83" s="53"/>
+      <c r="B83" s="54"/>
       <c r="C83" s="1" t="s">
         <v>380</v>
       </c>
@@ -4448,12 +4474,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="41"/>
-      <c r="B84" s="53"/>
+      <c r="B84" s="54"/>
       <c r="E84" s="2"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="41"/>
       <c r="B85" s="46" t="s">
         <v>4</v>
@@ -4469,7 +4495,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="41"/>
       <c r="B86" s="44"/>
       <c r="C86" s="1" t="s">
@@ -4483,7 +4509,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="41"/>
       <c r="B87" s="44"/>
       <c r="C87" s="1" t="s">
@@ -4497,7 +4523,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="41"/>
       <c r="B88" s="44"/>
       <c r="C88" s="1" t="s">
@@ -4511,7 +4537,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="41"/>
       <c r="B89" s="44"/>
       <c r="C89" s="1" t="s">
@@ -4525,7 +4551,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="41"/>
       <c r="B90" s="44"/>
       <c r="C90" s="1" t="s">
@@ -4539,7 +4565,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" s="41"/>
       <c r="B91" s="44"/>
       <c r="C91" s="1" t="s">
@@ -4553,7 +4579,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="41"/>
       <c r="B92" s="44"/>
       <c r="C92" s="1" t="s">
@@ -4567,7 +4593,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" s="41"/>
       <c r="B93" s="44"/>
       <c r="C93" s="1" t="s">
@@ -4581,11 +4607,11 @@
         <v>149</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="41"/>
       <c r="B94" s="45"/>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" s="41"/>
       <c r="B95" s="46" t="s">
         <v>5</v>
@@ -4601,7 +4627,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="41"/>
       <c r="B96" s="44"/>
       <c r="C96" s="1" t="s">
@@ -4615,7 +4641,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" s="41"/>
       <c r="B97" s="44"/>
       <c r="C97" s="1" t="s">
@@ -4629,7 +4655,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="41"/>
       <c r="B98" s="44"/>
       <c r="C98" s="1" t="s">
@@ -4643,7 +4669,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" s="41"/>
       <c r="B99" s="44"/>
       <c r="C99" s="1" t="s">
@@ -4657,7 +4683,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="41"/>
       <c r="B100" s="44"/>
       <c r="C100" s="1" t="s">
@@ -4671,7 +4697,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" s="41"/>
       <c r="B101" s="44"/>
       <c r="C101" s="1" t="s">
@@ -4685,7 +4711,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" s="41"/>
       <c r="B102" s="44"/>
       <c r="C102" s="1" t="s">
@@ -4699,7 +4725,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" s="41"/>
       <c r="B103" s="44"/>
       <c r="C103" s="1" t="s">
@@ -4713,11 +4739,11 @@
         <v>149</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="42"/>
       <c r="B104" s="47"/>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" s="40" t="s">
         <v>76</v>
       </c>
@@ -4735,7 +4761,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" s="41"/>
       <c r="B106" s="48"/>
       <c r="C106" s="1" t="s">
@@ -4749,7 +4775,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" s="41"/>
       <c r="B107" s="52"/>
       <c r="C107" s="17"/>
@@ -4757,7 +4783,7 @@
       <c r="E107" s="18"/>
       <c r="F107" s="17"/>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" s="41"/>
       <c r="B108" s="51" t="s">
         <v>263</v>
@@ -4773,7 +4799,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" s="41"/>
       <c r="B109" s="48"/>
       <c r="C109" s="1" t="s">
@@ -4787,12 +4813,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="41"/>
       <c r="B110" s="52"/>
       <c r="E110" s="3"/>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" s="41"/>
       <c r="B111" s="51" t="s">
         <v>79</v>
@@ -4808,7 +4834,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" s="41"/>
       <c r="B112" s="48"/>
       <c r="C112" s="1" t="s">
@@ -4822,7 +4848,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" s="41"/>
       <c r="B113" s="52"/>
       <c r="C113" s="17"/>
@@ -4830,7 +4856,7 @@
       <c r="E113" s="18"/>
       <c r="F113" s="17"/>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" s="41"/>
       <c r="B114" s="51" t="s">
         <v>340</v>
@@ -4846,7 +4872,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" s="41"/>
       <c r="B115" s="48"/>
       <c r="C115" s="1" t="s">
@@ -4860,7 +4886,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" s="41"/>
       <c r="B116" s="52"/>
       <c r="C116" s="17"/>
@@ -4868,7 +4894,7 @@
       <c r="E116" s="18"/>
       <c r="F116" s="17"/>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" s="41"/>
       <c r="B117" s="48" t="s">
         <v>300</v>
@@ -4884,7 +4910,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" s="41"/>
       <c r="B118" s="48"/>
       <c r="C118" s="1" t="s">
@@ -4898,7 +4924,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="42"/>
       <c r="B119" s="49"/>
       <c r="C119" s="27"/>
@@ -4906,7 +4932,7 @@
       <c r="E119" s="28"/>
       <c r="F119" s="27"/>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" s="40" t="s">
         <v>163</v>
       </c>
@@ -4924,7 +4950,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" s="41"/>
       <c r="B121" s="48"/>
       <c r="C121" s="1" t="s">
@@ -4937,7 +4963,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" s="41"/>
       <c r="B122" s="52"/>
       <c r="C122" s="17"/>
@@ -4945,7 +4971,7 @@
       <c r="E122" s="17"/>
       <c r="F122" s="17"/>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" s="41"/>
       <c r="B123" s="51" t="s">
         <v>183</v>
@@ -4960,7 +4986,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" s="41"/>
       <c r="B124" s="48"/>
       <c r="C124" s="1" t="s">
@@ -4973,7 +4999,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" s="41"/>
       <c r="B125" s="48"/>
       <c r="C125" s="1" t="s">
@@ -4986,7 +5012,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" s="41"/>
       <c r="B126" s="48"/>
       <c r="C126" s="1" t="s">
@@ -4999,7 +5025,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" s="41"/>
       <c r="B127" s="48"/>
       <c r="C127" s="1" t="s">
@@ -5012,7 +5038,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" s="41"/>
       <c r="B128" s="48"/>
       <c r="C128" s="1" t="s">
@@ -5025,11 +5051,11 @@
         <v>149</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" s="41"/>
       <c r="B129" s="52"/>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" s="41"/>
       <c r="B130" s="51" t="s">
         <v>206</v>
@@ -5045,7 +5071,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" s="41"/>
       <c r="B131" s="48"/>
       <c r="C131" s="1" t="s">
@@ -5058,7 +5084,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" s="41"/>
       <c r="B132" s="48"/>
       <c r="C132" s="1" t="s">
@@ -5071,7 +5097,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" s="41"/>
       <c r="B133" s="48"/>
       <c r="C133" s="1" t="s">
@@ -5084,7 +5110,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" s="41"/>
       <c r="B134" s="48"/>
       <c r="C134" s="1" t="s">
@@ -5097,7 +5123,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" s="41"/>
       <c r="B135" s="48"/>
       <c r="C135" s="1" t="s">
@@ -5110,7 +5136,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" s="41"/>
       <c r="B136" s="48"/>
       <c r="C136" s="1" t="s">
@@ -5123,7 +5149,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" s="41"/>
       <c r="B137" s="48"/>
       <c r="C137" s="1" t="s">
@@ -5136,7 +5162,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" s="41"/>
       <c r="B138" s="48"/>
       <c r="C138" s="1" t="s">
@@ -5149,7 +5175,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" s="41"/>
       <c r="B139" s="48"/>
       <c r="C139" s="1" t="s">
@@ -5162,7 +5188,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" s="41"/>
       <c r="B140" s="48"/>
       <c r="C140" s="1" t="s">
@@ -5175,7 +5201,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" s="41"/>
       <c r="B141" s="48"/>
       <c r="C141" s="1" t="s">
@@ -5188,7 +5214,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" s="41"/>
       <c r="B142" s="48"/>
       <c r="C142" s="1" t="s">
@@ -5201,7 +5227,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" s="41"/>
       <c r="B143" s="48"/>
       <c r="C143" s="1" t="s">
@@ -5214,11 +5240,11 @@
         <v>213</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" s="41"/>
       <c r="B144" s="52"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" s="41"/>
       <c r="B145" s="51" t="s">
         <v>222</v>
@@ -5234,7 +5260,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" s="41"/>
       <c r="B146" s="48"/>
       <c r="C146" s="1" t="s">
@@ -5247,7 +5273,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" s="41"/>
       <c r="B147" s="48"/>
       <c r="C147" s="1" t="s">
@@ -5260,7 +5286,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" s="41"/>
       <c r="B148" s="48"/>
       <c r="C148" s="1" t="s">
@@ -5273,7 +5299,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149" s="41"/>
       <c r="B149" s="48"/>
       <c r="C149" s="1" t="s">
@@ -5286,7 +5312,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150" s="41"/>
       <c r="B150" s="52"/>
       <c r="C150" s="17"/>
@@ -5294,9 +5320,9 @@
       <c r="E150" s="17"/>
       <c r="F150" s="17"/>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151" s="41"/>
-      <c r="B151" s="54" t="s">
+      <c r="B151" s="53" t="s">
         <v>355</v>
       </c>
       <c r="C151" s="1" t="s">
@@ -5309,9 +5335,9 @@
         <v>314</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152" s="41"/>
-      <c r="B152" s="54"/>
+      <c r="B152" s="53"/>
       <c r="C152" s="1" t="s">
         <v>357</v>
       </c>
@@ -5324,12 +5350,15 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B145:B150"/>
-    <mergeCell ref="B151:B152"/>
-    <mergeCell ref="A120:A152"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B130:B144"/>
-    <mergeCell ref="B123:B129"/>
+    <mergeCell ref="A2:A46"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B23"/>
+    <mergeCell ref="A47:A78"/>
+    <mergeCell ref="B67:B78"/>
+    <mergeCell ref="B24:B33"/>
+    <mergeCell ref="B47:B56"/>
+    <mergeCell ref="B57:B66"/>
+    <mergeCell ref="B34:B46"/>
     <mergeCell ref="B117:B119"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="A79:A104"/>
@@ -5341,15 +5370,12 @@
     <mergeCell ref="B111:B113"/>
     <mergeCell ref="B114:B116"/>
     <mergeCell ref="B82:B84"/>
-    <mergeCell ref="A2:A46"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B23"/>
-    <mergeCell ref="A47:A78"/>
-    <mergeCell ref="B67:B78"/>
-    <mergeCell ref="B24:B33"/>
-    <mergeCell ref="B47:B56"/>
-    <mergeCell ref="B57:B66"/>
-    <mergeCell ref="B34:B46"/>
+    <mergeCell ref="B145:B150"/>
+    <mergeCell ref="B151:B152"/>
+    <mergeCell ref="A120:A152"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B130:B144"/>
+    <mergeCell ref="B123:B129"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>